<commit_message>
state: bot run 2026-09-07T21:19 IST
</commit_message>
<xml_diff>
--- a/data/trade_log.xlsx
+++ b/data/trade_log.xlsx
@@ -431,61 +431,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SMA20</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Upper_Band</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Vol_Ratio</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Qualifies</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Rejection_Or_Status</t>
         </is>
@@ -2147,6 +2147,565 @@
       <c r="K40" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 1322.00 &lt;= Upper 1338.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>2814.5</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3029</v>
+      </c>
+      <c r="F41" t="n">
+        <v>3029</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2860.49</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2903.68</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J41" t="b">
+        <v>0</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2860.49 &lt;= EMA21 2903.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>404</v>
+      </c>
+      <c r="E42" t="n">
+        <v>415.89</v>
+      </c>
+      <c r="F42" t="n">
+        <v>415.89</v>
+      </c>
+      <c r="G42" t="n">
+        <v>407.85</v>
+      </c>
+      <c r="H42" t="n">
+        <v>407.67</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J42" t="b">
+        <v>0</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 404.00 &lt;= Upper 415.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>4855.2</v>
+      </c>
+      <c r="E43" t="n">
+        <v>5108.33</v>
+      </c>
+      <c r="F43" t="n">
+        <v>5108.33</v>
+      </c>
+      <c r="G43" t="n">
+        <v>4844.13</v>
+      </c>
+      <c r="H43" t="n">
+        <v>4842.43</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4855.20 &lt;= Upper 5108.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PERSISTENT</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>5540</v>
+      </c>
+      <c r="E44" t="n">
+        <v>5829.07</v>
+      </c>
+      <c r="F44" t="n">
+        <v>5829.07</v>
+      </c>
+      <c r="G44" t="n">
+        <v>5644.06</v>
+      </c>
+      <c r="H44" t="n">
+        <v>5591.91</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J44" t="b">
+        <v>0</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5540.00 &lt;= Upper 5829.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>DIXON</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>14180</v>
+      </c>
+      <c r="E45" t="n">
+        <v>15126.99</v>
+      </c>
+      <c r="F45" t="n">
+        <v>15126.99</v>
+      </c>
+      <c r="G45" t="n">
+        <v>14447.02</v>
+      </c>
+      <c r="H45" t="n">
+        <v>14390.89</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J45" t="b">
+        <v>0</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 14180.00 &lt;= Upper 15126.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1854</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2002.01</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2002.01</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1869.91</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1894.43</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J46" t="b">
+        <v>0</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1869.91 &lt;= EMA21 1894.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MCX</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3330.2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>3502.16</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3502.16</v>
+      </c>
+      <c r="G47" t="n">
+        <v>3264.29</v>
+      </c>
+      <c r="H47" t="n">
+        <v>3150.45</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J47" t="b">
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3330.20 &lt;= Upper 3502.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1848.2</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1928.55</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1928.55</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1848.48</v>
+      </c>
+      <c r="H48" t="n">
+        <v>1852.84</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J48" t="b">
+        <v>0</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1848.48 &lt;= EMA21 1852.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>710.5</v>
+      </c>
+      <c r="E49" t="n">
+        <v>738.1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>738.1</v>
+      </c>
+      <c r="G49" t="n">
+        <v>712.6900000000001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>721.96</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J49" t="b">
+        <v>0</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 712.69 &lt;= EMA21 721.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1427.5</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1448.8</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1448.8</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1428.85</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1426.34</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1427.50 &lt;= Upper 1448.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>POLYCAB</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>8261</v>
+      </c>
+      <c r="E51" t="n">
+        <v>9639.790000000001</v>
+      </c>
+      <c r="F51" t="n">
+        <v>9639.790000000001</v>
+      </c>
+      <c r="G51" t="n">
+        <v>8742.459999999999</v>
+      </c>
+      <c r="H51" t="n">
+        <v>8943.15</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J51" t="b">
+        <v>0</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8742.46 &lt;= EMA21 8943.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>405.95</v>
+      </c>
+      <c r="E52" t="n">
+        <v>452.16</v>
+      </c>
+      <c r="F52" t="n">
+        <v>452.16</v>
+      </c>
+      <c r="G52" t="n">
+        <v>412.35</v>
+      </c>
+      <c r="H52" t="n">
+        <v>423.55</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J52" t="b">
+        <v>0</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 412.35 &lt;= EMA21 423.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1309.5</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1336.85</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1336.85</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1306.79</v>
+      </c>
+      <c r="H53" t="n">
+        <v>1306.32</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J53" t="b">
+        <v>0</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1309.50 &lt;= Upper 1336.85)</t>
         </is>
       </c>
     </row>
@@ -2216,57 +2775,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Unrealized_PnL_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Hard_SL</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Highest_High</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -2287,67 +2846,67 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Entry_Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Exit_Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Entry_Price</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Exit_Price</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Gross_PnL_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Net_PnL_Pct</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>PnL_Amount</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Exit_Reason</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Days_Held</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -3184,57 +3743,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Expected_Price</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Fill_Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Slippage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -8239,27 +8798,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Details</t>
         </is>
@@ -8303,51 +8862,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Cash_Available</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Invested_Capital</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total_Equity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Realized_PnL</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Win_Rate_Pct</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Total_Trades</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Open_Positions</t>
         </is>
@@ -8449,6 +9008,39 @@
         <v>17</v>
       </c>
       <c r="I4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>21:19:22</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>198821.93</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1092.43</v>
+      </c>
+      <c r="G5" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>17</v>
+      </c>
+      <c r="I5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>